<commit_message>
Refresh README and add dataset tooling & metadata
- Streamline the README around downloading and using the dataset; move CAD
  regeneration into an optional "Reproducing or Extending" section and reduce
  validation to a short quality summary.
- Add the 48 SolidWorks design tables (cad2ply/design_tables/) with per-instance
  CAD and defect parameters.
- Add metadata/normalization_params.csv to recover millimeter coordinates
  (p_mm = s*p_norm + c) from the normalized point clouds.
- point_sampling.py: 100k default, unit-sphere normalized by default, with
  --no-normalize for mm output and --num_points for arbitrary density.
- Provide the SolidWorks export macro as sanitized text (saveply251.bas).
- Add reconstruct_gear.py and document the validation tooling.
- Remove duplicate design tables; strip local paths and author metadata from
  published files.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cad2ply/gear_basemodels.xlsx
+++ b/cad2ply/gear_basemodels.xlsx
@@ -4,9 +4,7 @@
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25629"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rsmei2\Box\ADML\point-cloud\data\raw\GearPartGen\"/>
-    </mc:Choice>
+    <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C59EB9D-5F74-4A52-B2B2-73032605F855}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>

</xml_diff>